<commit_message>
chore: ajustar colores de texto en la plantilla
</commit_message>
<xml_diff>
--- a/storage/plantilla_test.xlsx
+++ b/storage/plantilla_test.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qwe\Documents\personal\senati\projects\practicas\sys_proforma\storage\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qwe\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D577480-F85D-4FCF-BDE5-1115C39639B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49FCEC4A-547E-45DF-A222-FB512A975F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -148,7 +148,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -247,46 +247,14 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="20"/>
-      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -417,7 +385,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -513,31 +481,59 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -550,72 +546,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="17" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="17" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3461,76 +3424,6 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>1228725</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>485775</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="CuadroTexto 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8DE3C23-32F6-C40C-6A52-58176915D771}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5800725" y="1228725"/>
-          <a:ext cx="914400" cy="914400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1100"/>
-            <a:t>hola prueba</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -3835,96 +3728,98 @@
   <sheetData>
     <row r="1" spans="1:10" ht="130.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:10" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="37" t="s">
+      <c r="B3" s="58"/>
+      <c r="C3" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="37"/>
-      <c r="E3" s="55" t="s">
+      <c r="D3" s="59"/>
+      <c r="E3" s="49" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="53"/>
-      <c r="C4" s="37" t="s">
+      <c r="B4" s="58"/>
+      <c r="C4" s="59" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="56" t="s">
+      <c r="D4" s="60"/>
+      <c r="E4" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="56"/>
-      <c r="G4" s="56"/>
-      <c r="H4" s="56"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="50"/>
     </row>
     <row r="5" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="54" t="s">
+      <c r="A5" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="54"/>
-      <c r="C5" s="36" t="s">
+      <c r="B5" s="51"/>
+      <c r="C5" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="57" t="s">
+      <c r="D5" s="60"/>
+      <c r="E5" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
+      <c r="F5" s="51"/>
+      <c r="G5" s="51"/>
+      <c r="H5" s="51"/>
     </row>
     <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="59" t="s">
+      <c r="A6" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="59"/>
-      <c r="C6" s="59"/>
-      <c r="D6" s="59"/>
+      <c r="B6" s="39"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="39"/>
       <c r="E6" s="5"/>
       <c r="F6" s="12"/>
       <c r="G6" s="5"/>
       <c r="H6" s="3"/>
     </row>
     <row r="7" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="67" t="s">
+      <c r="C7" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="68"/>
-      <c r="E7" s="39" t="s">
+      <c r="D7" s="63"/>
+      <c r="E7" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="39" t="s">
+      <c r="F7" s="61" t="s">
         <v>23</v>
       </c>
-      <c r="G7" s="40" t="s">
+      <c r="G7" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="H7" s="41" t="s">
+      <c r="H7" s="65" t="s">
         <v>2</v>
       </c>
     </row>
@@ -3933,8 +3828,8 @@
         <v>1</v>
       </c>
       <c r="B8" s="24"/>
-      <c r="C8" s="69"/>
-      <c r="D8" s="70"/>
+      <c r="C8" s="45"/>
+      <c r="D8" s="46"/>
       <c r="E8" s="29"/>
       <c r="F8" s="29"/>
       <c r="G8" s="34"/>
@@ -3945,8 +3840,8 @@
         <v>2</v>
       </c>
       <c r="B9" s="24"/>
-      <c r="C9" s="69"/>
-      <c r="D9" s="70"/>
+      <c r="C9" s="45"/>
+      <c r="D9" s="46"/>
       <c r="E9" s="29"/>
       <c r="F9" s="29"/>
       <c r="G9" s="34"/>
@@ -3958,8 +3853,8 @@
         <v>3</v>
       </c>
       <c r="B10" s="24"/>
-      <c r="C10" s="69"/>
-      <c r="D10" s="70"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="46"/>
       <c r="E10" s="29"/>
       <c r="F10" s="29"/>
       <c r="G10" s="34"/>
@@ -3971,8 +3866,8 @@
         <v>4</v>
       </c>
       <c r="B11" s="30"/>
-      <c r="C11" s="50"/>
-      <c r="D11" s="51"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="48"/>
       <c r="E11" s="29"/>
       <c r="F11" s="29"/>
       <c r="G11" s="23"/>
@@ -3983,8 +3878,8 @@
         <v>5</v>
       </c>
       <c r="B12" s="30"/>
-      <c r="C12" s="50"/>
-      <c r="D12" s="51"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="48"/>
       <c r="E12" s="29"/>
       <c r="F12" s="29"/>
       <c r="G12" s="23"/>
@@ -3995,8 +3890,8 @@
         <v>6</v>
       </c>
       <c r="B13" s="30"/>
-      <c r="C13" s="50"/>
-      <c r="D13" s="51"/>
+      <c r="C13" s="47"/>
+      <c r="D13" s="48"/>
       <c r="E13" s="29"/>
       <c r="F13" s="29"/>
       <c r="G13" s="23"/>
@@ -4007,8 +3902,8 @@
         <v>7</v>
       </c>
       <c r="B14" s="30"/>
-      <c r="C14" s="50"/>
-      <c r="D14" s="51"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="48"/>
       <c r="E14" s="29"/>
       <c r="F14" s="29"/>
       <c r="G14" s="23"/>
@@ -4019,8 +3914,8 @@
         <v>8</v>
       </c>
       <c r="B15" s="30"/>
-      <c r="C15" s="50"/>
-      <c r="D15" s="51"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="48"/>
       <c r="E15" s="29"/>
       <c r="F15" s="29"/>
       <c r="G15" s="23"/>
@@ -4031,8 +3926,8 @@
         <v>9</v>
       </c>
       <c r="B16" s="30"/>
-      <c r="C16" s="50"/>
-      <c r="D16" s="51"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="48"/>
       <c r="E16" s="29"/>
       <c r="F16" s="29"/>
       <c r="G16" s="23"/>
@@ -4043,8 +3938,8 @@
         <v>10</v>
       </c>
       <c r="B17" s="30"/>
-      <c r="C17" s="50"/>
-      <c r="D17" s="51"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="48"/>
       <c r="E17" s="29"/>
       <c r="F17" s="29"/>
       <c r="G17" s="23"/>
@@ -4055,8 +3950,8 @@
         <v>11</v>
       </c>
       <c r="B18" s="30"/>
-      <c r="C18" s="50"/>
-      <c r="D18" s="51"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="48"/>
       <c r="E18" s="29"/>
       <c r="F18" s="29"/>
       <c r="G18" s="23"/>
@@ -4067,8 +3962,8 @@
         <v>12</v>
       </c>
       <c r="B19" s="30"/>
-      <c r="C19" s="50"/>
-      <c r="D19" s="51"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="48"/>
       <c r="E19" s="29"/>
       <c r="F19" s="29"/>
       <c r="G19" s="23"/>
@@ -4079,8 +3974,8 @@
         <v>13</v>
       </c>
       <c r="B20" s="30"/>
-      <c r="C20" s="50"/>
-      <c r="D20" s="51"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="48"/>
       <c r="E20" s="29"/>
       <c r="F20" s="29"/>
       <c r="G20" s="23"/>
@@ -4091,8 +3986,8 @@
         <v>14</v>
       </c>
       <c r="B21" s="30"/>
-      <c r="C21" s="50"/>
-      <c r="D21" s="51"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="48"/>
       <c r="E21" s="29"/>
       <c r="F21" s="29"/>
       <c r="G21" s="23"/>
@@ -4103,8 +3998,8 @@
         <v>15</v>
       </c>
       <c r="B22" s="30"/>
-      <c r="C22" s="50"/>
-      <c r="D22" s="51"/>
+      <c r="C22" s="47"/>
+      <c r="D22" s="48"/>
       <c r="E22" s="29"/>
       <c r="F22" s="29"/>
       <c r="G22" s="23"/>
@@ -4115,8 +4010,8 @@
         <v>16</v>
       </c>
       <c r="B23" s="30"/>
-      <c r="C23" s="50"/>
-      <c r="D23" s="51"/>
+      <c r="C23" s="47"/>
+      <c r="D23" s="48"/>
       <c r="E23" s="29"/>
       <c r="F23" s="29"/>
       <c r="G23" s="23"/>
@@ -4127,8 +4022,8 @@
         <v>17</v>
       </c>
       <c r="B24" s="30"/>
-      <c r="C24" s="50"/>
-      <c r="D24" s="51"/>
+      <c r="C24" s="47"/>
+      <c r="D24" s="48"/>
       <c r="E24" s="33"/>
       <c r="F24" s="29"/>
       <c r="G24" s="23"/>
@@ -4139,8 +4034,8 @@
         <v>18</v>
       </c>
       <c r="B25" s="28"/>
-      <c r="C25" s="48"/>
-      <c r="D25" s="49"/>
+      <c r="C25" s="52"/>
+      <c r="D25" s="53"/>
       <c r="E25" s="33"/>
       <c r="F25" s="29"/>
       <c r="G25" s="23"/>
@@ -4151,8 +4046,8 @@
         <v>19</v>
       </c>
       <c r="B26" s="28"/>
-      <c r="C26" s="48"/>
-      <c r="D26" s="49"/>
+      <c r="C26" s="52"/>
+      <c r="D26" s="53"/>
       <c r="E26" s="33"/>
       <c r="F26" s="29"/>
       <c r="G26" s="23"/>
@@ -4163,8 +4058,8 @@
         <v>20</v>
       </c>
       <c r="B27" s="28"/>
-      <c r="C27" s="48"/>
-      <c r="D27" s="49"/>
+      <c r="C27" s="52"/>
+      <c r="D27" s="53"/>
       <c r="E27" s="25"/>
       <c r="F27" s="25"/>
       <c r="G27" s="19"/>
@@ -4175,8 +4070,8 @@
         <v>21</v>
       </c>
       <c r="B28" s="28"/>
-      <c r="C28" s="48"/>
-      <c r="D28" s="49"/>
+      <c r="C28" s="52"/>
+      <c r="D28" s="53"/>
       <c r="E28" s="25"/>
       <c r="F28" s="25"/>
       <c r="G28" s="19"/>
@@ -4187,8 +4082,8 @@
         <v>22</v>
       </c>
       <c r="B29" s="28"/>
-      <c r="C29" s="48"/>
-      <c r="D29" s="49"/>
+      <c r="C29" s="52"/>
+      <c r="D29" s="53"/>
       <c r="E29" s="25"/>
       <c r="F29" s="25"/>
       <c r="G29" s="19"/>
@@ -4199,8 +4094,8 @@
         <v>23</v>
       </c>
       <c r="B30" s="28"/>
-      <c r="C30" s="48"/>
-      <c r="D30" s="49"/>
+      <c r="C30" s="52"/>
+      <c r="D30" s="53"/>
       <c r="E30" s="25"/>
       <c r="F30" s="25"/>
       <c r="G30" s="19"/>
@@ -4211,8 +4106,8 @@
         <v>24</v>
       </c>
       <c r="B31" s="28"/>
-      <c r="C31" s="48"/>
-      <c r="D31" s="49"/>
+      <c r="C31" s="52"/>
+      <c r="D31" s="53"/>
       <c r="E31" s="25"/>
       <c r="F31" s="25"/>
       <c r="G31" s="19"/>
@@ -4223,8 +4118,8 @@
         <v>25</v>
       </c>
       <c r="B32" s="28"/>
-      <c r="C32" s="48"/>
-      <c r="D32" s="49"/>
+      <c r="C32" s="52"/>
+      <c r="D32" s="53"/>
       <c r="E32" s="26"/>
       <c r="F32" s="17"/>
       <c r="G32" s="19"/>
@@ -4235,8 +4130,8 @@
         <v>26</v>
       </c>
       <c r="B33" s="16"/>
-      <c r="C33" s="44"/>
-      <c r="D33" s="45"/>
+      <c r="C33" s="54"/>
+      <c r="D33" s="55"/>
       <c r="E33" s="20"/>
       <c r="F33" s="20"/>
       <c r="G33" s="20"/>
@@ -4247,8 +4142,8 @@
         <v>27</v>
       </c>
       <c r="B34" s="16"/>
-      <c r="C34" s="44"/>
-      <c r="D34" s="45"/>
+      <c r="C34" s="54"/>
+      <c r="D34" s="55"/>
       <c r="E34" s="16"/>
       <c r="F34" s="17"/>
       <c r="G34" s="19"/>
@@ -4259,8 +4154,8 @@
         <v>28</v>
       </c>
       <c r="B35" s="31"/>
-      <c r="C35" s="44"/>
-      <c r="D35" s="45"/>
+      <c r="C35" s="54"/>
+      <c r="D35" s="55"/>
       <c r="E35" s="20"/>
       <c r="F35" s="20"/>
       <c r="G35" s="20"/>
@@ -4271,8 +4166,8 @@
         <v>29</v>
       </c>
       <c r="B36" s="31"/>
-      <c r="C36" s="44"/>
-      <c r="D36" s="45"/>
+      <c r="C36" s="54"/>
+      <c r="D36" s="55"/>
       <c r="E36" s="20"/>
       <c r="F36" s="20"/>
       <c r="G36" s="20"/>
@@ -4283,8 +4178,8 @@
         <v>30</v>
       </c>
       <c r="B37" s="22"/>
-      <c r="C37" s="46"/>
-      <c r="D37" s="47"/>
+      <c r="C37" s="56"/>
+      <c r="D37" s="57"/>
       <c r="E37" s="20"/>
       <c r="F37" s="20"/>
       <c r="G37" s="20"/>
@@ -4292,11 +4187,11 @@
     </row>
     <row r="38" spans="1:8" s="6" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="8"/>
-      <c r="B38" s="58" t="s">
+      <c r="B38" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="C38" s="58"/>
-      <c r="D38" s="58"/>
+      <c r="C38" s="66"/>
+      <c r="D38" s="66"/>
       <c r="E38"/>
       <c r="F38" s="14" t="s">
         <v>3</v>
@@ -4310,13 +4205,13 @@
     </row>
     <row r="39" spans="1:8" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
-      <c r="B39" s="63" t="s">
+      <c r="B39" s="67" t="s">
         <v>11</v>
       </c>
-      <c r="C39" s="63"/>
-      <c r="D39" s="63"/>
+      <c r="C39" s="67"/>
+      <c r="D39" s="67"/>
       <c r="E39"/>
-      <c r="F39" s="35">
+      <c r="F39" s="7">
         <f>SUM(H8:H19)</f>
         <v>0</v>
       </c>
@@ -4324,18 +4219,18 @@
         <f>F39*0.18</f>
         <v>0</v>
       </c>
-      <c r="H39" s="35">
+      <c r="H39" s="7">
         <f>G39+F39</f>
         <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="64" t="s">
+      <c r="B40" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="C40" s="64"/>
-      <c r="D40" s="64"/>
+      <c r="C40" s="42"/>
+      <c r="D40" s="42"/>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
@@ -4343,25 +4238,25 @@
     </row>
     <row r="41" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
-      <c r="B41" s="65" t="s">
+      <c r="B41" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="C41" s="65"/>
-      <c r="D41" s="43" t="s">
+      <c r="C41" s="43"/>
+      <c r="D41" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="E41" s="61"/>
-      <c r="F41" s="61"/>
-      <c r="G41" s="61"/>
-      <c r="H41" s="61"/>
+      <c r="E41" s="41"/>
+      <c r="F41" s="41"/>
+      <c r="G41" s="41"/>
+      <c r="H41" s="41"/>
     </row>
     <row r="42" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
-      <c r="B42" s="66" t="s">
+      <c r="B42" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="C42" s="66"/>
-      <c r="D42" s="42" t="s">
+      <c r="C42" s="44"/>
+      <c r="D42" s="36" t="s">
         <v>29</v>
       </c>
       <c r="E42" s="9"/>
@@ -4412,12 +4307,12 @@
       <c r="B47"/>
       <c r="C47"/>
       <c r="D47" s="1"/>
-      <c r="E47" s="62" t="s">
+      <c r="E47" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="F47" s="62"/>
-      <c r="G47" s="62"/>
-      <c r="H47" s="62"/>
+      <c r="F47" s="68"/>
+      <c r="G47" s="68"/>
+      <c r="H47" s="68"/>
     </row>
     <row r="48" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48"/>
@@ -4432,16 +4327,16 @@
       <c r="H48" s="1"/>
     </row>
     <row r="49" spans="1:8" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A49" s="60" t="s">
+      <c r="A49" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="B49" s="60"/>
-      <c r="C49" s="60"/>
-      <c r="D49" s="60"/>
-      <c r="E49" s="60"/>
-      <c r="F49" s="60"/>
-      <c r="G49" s="60"/>
-      <c r="H49" s="60"/>
+      <c r="B49" s="40"/>
+      <c r="C49" s="40"/>
+      <c r="D49" s="40"/>
+      <c r="E49" s="40"/>
+      <c r="F49" s="40"/>
+      <c r="G49" s="40"/>
+      <c r="H49" s="40"/>
     </row>
     <row r="50" spans="1:8" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="E50" s="4"/>
@@ -4685,6 +4580,37 @@
     </row>
   </sheetData>
   <mergeCells count="47">
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="E5:H5"/>
     <mergeCell ref="B38:D38"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A49:H49"/>
@@ -4701,37 +4627,6 @@
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="C13:D13"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C33:D33"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.11811023622047245" right="0.11811023622047245" top="0.43307086614173229" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.23622047244094491"/>

</xml_diff>